<commit_message>
Timesheet: add 26-27 Aug entries
Seven entries covering the live-system research, the customer's Testing
Guideline, the corrections it forced, and the completion of both Project
Requirements views.

Split across two days on a natural boundary — research and form view on the
26th, list view and documentation on the 27th. Hours are a scope estimate, not
a clock reading, and need reconciling against the actual record before invoicing.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Voyager-UIUX-Timesheet-Aug2026.xlsx
+++ b/docs/Voyager-UIUX-Timesheet-Aug2026.xlsx
@@ -769,7 +769,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:D49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1435,6 +1435,157 @@
         <is>
           <t>•  Current phase covers layout and user experience. Visual design — colour, spacing, typography and component styling — is a later phase, so that it is not done twice.</t>
         </is>
+      </c>
+    </row>
+    <row r="42" ht="62" customHeight="1">
+      <c r="A42" s="16" t="inlineStr">
+        <is>
+          <t>26/08/2026</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Live system research, signed in. Walked the real system and recorded how it actually behaves — the filter panel, the saved-view settings and its three tabs, every field on the RFQ form, the true option values and the page numbering. Written up as a verified reference so later work is checked against fact rather than memory.</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Deliverable: verified reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="62" customHeight="1">
+      <c r="A43" s="16" t="inlineStr">
+        <is>
+          <t>26/08/2026</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Received and catalogued the client's Testing Guideline. Extracted all fifteen sheets into a readable reference and saved both files to the project. This document turns out to be the functional specification, so it now outranks the running system wherever the two disagree.</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Client document</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="62" customHeight="1">
+      <c r="A44" s="16" t="inlineStr">
+        <is>
+          <t>26/08/2026</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Corrections the guideline forced. Required markers changed to red as specified; Historical RFQ restored after being wrongly removed — it appears only when Order Type is Repeat, so it was correctly hidden on the one record checked.</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Correction</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="62" customHeight="1">
+      <c r="A45" s="16" t="inlineStr">
+        <is>
+          <t>26/08/2026</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Form view completed. Real tab and section names restored, required markers added to nineteen fields, three fields removed that do not exist on the real form, option values corrected and shown as radio choices with their meanings, ITAR built as the access-control rule it actually is, required-field validation added, Quotation Result columns corrected, and the Conversations tab rebuilt with its Comment / Send Email choice and full text editor.</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>6</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Fidelity + build</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="62" customHeight="1">
+      <c r="A46" s="16" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>List view completed. Real columns in the real order, View Detail action restored, page sizes and wording matched, first and last page navigation added, the filter rebuilt as the real one — every field at once, no operators — and saved views built with the View Setting sidebar: choose filter fields, reorder and rename columns, set widths, and stack multiple sort levels.</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Fidelity + build</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="62" customHeight="1">
+      <c r="A47" s="16" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Defects found and fixed while checking. Quoted status badges had been rendering with no colour at all; a column was too narrow for its longest value and made rows uneven; and an empty grid gave the wrong advice, blaming the search when filters were responsible.</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Defect fixing</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="44" customHeight="1">
+      <c r="A48" s="16" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Client documentation. Prepared the KendoReact licence activation document answering how activation works through npm and what is needed from the client, and this timesheet.</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Deliverable: client document</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C49">
+        <f>SUM(C6:C48)</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>